<commit_message>
Correct ten points in the survey design case study
The raw numbers understate support by about 7 points without reversing the majority. Treating design weights as counts acts as if the sample were the 38,693 the weights sum to, uniform response rates keep the district mix intact, and DescrStatsW gives the mean and SD while the interval uses the Kish effective n, which is slightly conservative here. A confirmatory survey with this design needs about 1,400 responses. Lakeside and Oldtown carry the smallest weights, and the workbook's Notes give 78% and Chapter 70.
</commit_message>
<xml_diff>
--- a/data/case-study-designing-and-analyzing-a-survey--survey.xlsx
+++ b/data/case-study-designing-and-analyzing-a-survey--survey.xlsx
@@ -30845,7 +30845,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Simulated survey for a stratified-sampling + estimation capstone (Chapter 136).</t>
+          <t>Simulated survey for a stratified-sampling + estimation capstone (Chapter 70).</t>
         </is>
       </c>
     </row>
@@ -30866,7 +30866,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Response is roughly uniform across districts (~76%); a small nonresponse-sensitivity check is left for the Take It Further notebook.</t>
+          <t>Response is roughly uniform across districts (~78%); a small nonresponse-sensitivity check is left for the Take It Further notebook.</t>
         </is>
       </c>
     </row>

</xml_diff>